<commit_message>
fix the `<src>` reference entry for `<frame>`, `<cover>` and `<audio>`
The `<src>` entry in the Reference still described it as the image's
source that can only appear in `<picture>`. Since #175, `<frame>`,
`<cover>` and `<audio>` take an optional `<src>` too, as the Tracks
section, the XSD (`media_capture_type`) and the valid track fixtures
already show.

- update the `<src>` row in reference/input/reference.xlsx
- regenerate the Reference section of spec.md

Signed-off-by: Daniel Nguyen <danielnguyenh07@gmail.com>
</commit_message>
<xml_diff>
--- a/reference/input/reference.xlsx
+++ b/reference/input/reference.xlsx
@@ -2041,12 +2041,12 @@
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>The image's source.</t>
+          <t>The source of the element's media: an image in `&lt;picture&gt;`, `&lt;frame&gt;` and `&lt;cover&gt;`, or an audio clip in `&lt;audio&gt;`.</t>
         </is>
       </c>
       <c r="D38" s="5" t="inlineStr">
         <is>
-          <t>Can only be part of the picture-specific element body sequence of `&lt;picture&gt;`.</t>
+          <t>Can only be part of the picture-specific element body sequence of `&lt;picture&gt;`, or come right after the element head of `&lt;frame&gt;`, `&lt;cover&gt;` or `&lt;audio&gt;`.</t>
         </is>
       </c>
       <c r="E38" s="6" t="b">

</xml_diff>

<commit_message>
fix `<src>` reference entry for `<frame>`, `<cover>` and `<audio>` (#199)
* fix the `<src>` reference entry for `<frame>`, `<cover>` and `<audio>`

The `<src>` entry in the Reference still described it as the image's
source that can only appear in `<picture>`. Since #175, `<frame>`,
`<cover>` and `<audio>` take an optional `<src>` too, as the Tracks
section, the XSD (`media_capture_type`) and the valid track fixtures
already show.

- update the `<src>` row in reference/input/reference.xlsx
- regenerate the Reference section of spec.md

Signed-off-by: Daniel Nguyen <danielnguyenh07@gmail.com>

* update the XSD comment for the `<src>` element

Signed-off-by: Panos Vagenas <pva@zurich.ibm.com>

---------

Signed-off-by: Daniel Nguyen <danielnguyenh07@gmail.com>
Signed-off-by: Panos Vagenas <pva@zurich.ibm.com>
Co-authored-by: Panos Vagenas <pva@zurich.ibm.com>
</commit_message>
<xml_diff>
--- a/reference/input/reference.xlsx
+++ b/reference/input/reference.xlsx
@@ -2041,12 +2041,12 @@
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>The image's source.</t>
+          <t>The source of the element's media: an image in `&lt;picture&gt;`, `&lt;frame&gt;` and `&lt;cover&gt;`, or an audio clip in `&lt;audio&gt;`.</t>
         </is>
       </c>
       <c r="D38" s="5" t="inlineStr">
         <is>
-          <t>Can only be part of the picture-specific element body sequence of `&lt;picture&gt;`.</t>
+          <t>Can only be part of the picture-specific element body sequence of `&lt;picture&gt;`, or come right after the element head of `&lt;frame&gt;`, `&lt;cover&gt;` or `&lt;audio&gt;`.</t>
         </is>
       </c>
       <c r="E38" s="6" t="b">

</xml_diff>

<commit_message>
reformat appendix into annexes (#187)
* reformat appendix into annexes

Signed-off-by: Arnaud J Le Hors <lehors@us.ibm.com>

* fix test_tokenization

Signed-off-by: Arnaud J Le Hors <lehors@us.ibm.com>

* use single-line annex headings and update links to them

Signed-off-by: Panos Vagenas <pva@zurich.ibm.com>

* resolve links to headings with punctuation in the Word export

Signed-off-by: Panos Vagenas <pva@zurich.ibm.com>

---------

Signed-off-by: Arnaud J Le Hors <lehors@us.ibm.com>
Signed-off-by: Panos Vagenas <pva@zurich.ibm.com>
Co-authored-by: Panos Vagenas <pva@zurich.ibm.com>
</commit_message>
<xml_diff>
--- a/reference/input/reference.xlsx
+++ b/reference/input/reference.xlsx
@@ -1182,7 +1182,7 @@
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>Captures a code snippet, either as a standalone block or inlined within a semantic element. For language classification, use a `&lt;label&gt;`in the element head (see [Recommendations](#recommendations)).</t>
+          <t>Captures a code snippet, either as a standalone block or inlined within a semantic element. For language classification, use a `&lt;label&gt;`in the element head (see [Recommendations](#annex-c-informative-recommendations)).</t>
         </is>
       </c>
       <c r="D15" s="5" t="inlineStr">
@@ -1858,7 +1858,7 @@
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>Optional part of the element head; custom metadata, e.g. for application-specific purposes. See [Recommendations](#recommendations) for naming and namespacing guidance for custom vocabularies.</t>
+          <t>Optional part of the element head; custom metadata, e.g. for application-specific purposes. See [Recommendations](#annex-c-informative-recommendations) for naming and namespacing guidance for custom vocabularies.</t>
         </is>
       </c>
       <c r="D33" s="6" t="inlineStr">

</xml_diff>

<commit_message>
describe table structure tokens in logical terms
The descriptions of `<lcel>`, `<ucel>`, `<xcel>` and `<corn>` used "left",
"above", "horizontally" and "vertically". This is only correct for a
left-to-right horizontal layout. Describe them by row and cell order, and
add a note to the Tables section on right-to-left and vertical tables.

Signed-off-by: Daniel Nguyen <danielnguyenh07@gmail.com>
</commit_message>
<xml_diff>
--- a/reference/input/reference.xlsx
+++ b/reference/input/reference.xlsx
@@ -2590,7 +2590,7 @@
       </c>
       <c r="C54" s="5" t="inlineStr">
         <is>
-          <t>Indicates the beginning of a corner cell, typically the top-left header intersection.</t>
+          <t>Indicates the beginning of a corner cell, typically where the column headers and the row headers meet.</t>
         </is>
       </c>
       <c r="D54" s="5" t="inlineStr">
@@ -2658,7 +2658,7 @@
       </c>
       <c r="C56" s="5" t="inlineStr">
         <is>
-          <t>Left-merge extension token; extends the previous cell horizontally (colspan continuation).</t>
+          <t>Left-merge extension token; extends the previous cell in the same row (colspan continuation).</t>
         </is>
       </c>
       <c r="D56" s="5" t="inlineStr">
@@ -2692,7 +2692,7 @@
       </c>
       <c r="C57" s="5" t="inlineStr">
         <is>
-          <t>Upward-merge extension token; extends the cell above vertically (rowspan continuation)</t>
+          <t>Upward-merge extension token; extends the cell at the same position in the previous row (rowspan continuation).</t>
         </is>
       </c>
       <c r="D57" s="5" t="inlineStr">
@@ -2726,7 +2726,7 @@
       </c>
       <c r="C58" s="5" t="inlineStr">
         <is>
-          <t>Cross/combined span extension token; used where both horizontal and vertical spanning intersect.</t>
+          <t>Cross/combined span extension token; used where a colspan continuation and a rowspan continuation intersect.</t>
         </is>
       </c>
       <c r="D58" s="5" t="inlineStr">

</xml_diff>

<commit_message>
add `<writing_mode>` for vertical layout
DocLang had no way to declare that lines are vertical, e.g. in Japanese or
Chinese text where lines run top to bottom and follow each other from right
to left.

Add `<writing_mode value="horizontal_tb|vertical_rl|vertical_lr"/>`. In
`<head>` it sets the document default. In an element head (after `<layer>`,
before `<location>`) it applies to the element and its descendants. Content
stays in reading order and `<location>` keeps its coordinate system.

Schematron allows at most one `<writing_mode>` in `<head>`. The migration
step drops the element, and the token vocabulary gets
`<writing_mode value="`.

Signed-off-by: Daniel Nguyen <danielnguyenh07@gmail.com>
</commit_message>
<xml_diff>
--- a/reference/input/reference.xlsx
+++ b/reference/input/reference.xlsx
@@ -620,7 +620,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J88"/>
+  <dimension ref="A1:J89"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="20" defaultRowHeight="16"/>
   <cols>
     <col width="27.1640625" bestFit="1" customWidth="1" style="2" min="1" max="1"/>
@@ -3967,6 +3967,43 @@
         <v>0</v>
       </c>
     </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>[03a] property (outer)</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>`&lt;writing_mode&gt;`</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>Optional part of the element head, or of the document head; declares the writing mode, i.e. whether lines are horizontal or vertical, and the direction in which lines follow each other. In `&lt;head&gt;`, it sets the default writing mode of the DocLang instance. In an element head, it sets the writing mode of the host element and of its descendants. An element without `&lt;writing_mode&gt;` takes the writing mode of its nearest ancestor that declares one, otherwise the default of the DocLang instance, otherwise "horizontal_tb". The writing mode does not change the order of the content, which is always the reading order, nor the coordinate system of `&lt;location&gt;`.</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>Can only be part of the [element head](#element-head) of a semantic element, or child of `&lt;head&gt;`.</t>
+        </is>
+      </c>
+      <c r="E89" t="b">
+        <v>0</v>
+      </c>
+      <c r="F89" t="b">
+        <v>0</v>
+      </c>
+      <c r="G89" t="b">
+        <v>0</v>
+      </c>
+      <c r="H89" t="b">
+        <v>0</v>
+      </c>
+      <c r="I89" t="b">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:H82"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3980,7 +4017,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E24"/>
+  <dimension ref="A1:E25"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col width="12.5" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -4633,6 +4670,33 @@
         </is>
       </c>
     </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>`&lt;writing_mode&gt;`</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>`value`</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>{"horizontal_tb", "vertical_rl", "vertical_lr"}</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>The writing mode: "horizontal_tb" for horizontal lines that follow each other from top to bottom; "vertical_rl" for vertical lines, read from top to bottom, that follow each other from right to left (e.g. traditional Japanese or Chinese); "vertical_lr" for vertical lines, read from top to bottom, that follow each other from left to right (e.g. traditional Mongolian). The values correspond to the CSS `writing-mode` values "horizontal-tb", "vertical-rl" and "vertical-lr" (see Bibliography [4]).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:E12"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>